<commit_message>
Added more doucmentation and changed to english language
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-conclusioncode-cs.xlsx
+++ b/docs/CodeSystem-retina-conclusioncode-cs.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Kodeverk for konklusjon etter KI-anlyse</t>
+    <t>Conclusion From External Client</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-11-08T17:39:22+01:00</t>
+    <t>2025-11-11T17:38:50+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Verdisett som beskriver verdier for forløpsstatus for neste undersøkelse for Retinascreening etter KI</t>
+    <t>Codes describing where the external client has landed in its assessment of the examination. (1000-series)</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -141,19 +141,19 @@
     <t>1001</t>
   </si>
   <si>
-    <t>Ferdig etter KI</t>
+    <t>Grading completed</t>
   </si>
   <si>
     <t>1002</t>
   </si>
   <si>
-    <t>Til manuell primærgradering etter KI</t>
+    <t>To primary grading</t>
   </si>
   <si>
     <t>1003</t>
   </si>
   <si>
-    <t>Til sekundærgradering etter KI</t>
+    <t>To secondary grading</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Change title and description on the code systems
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-conclusioncode-cs.xlsx
+++ b/docs/CodeSystem-retina-conclusioncode-cs.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Conclusion From External Client</t>
+    <t>Grading Conclusion</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-11-11T17:38:50+01:00</t>
+    <t>2025-11-12T18:21:01+01:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Add videre-forlop-extension with cods from videre-forlop-cs to examples. Chagnge some titles.
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-conclusioncode-cs.xlsx
+++ b/docs/CodeSystem-retina-conclusioncode-cs.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Conclusion From External Client</t>
+    <t>Grading Conclusion</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-11-11T17:38:50+01:00</t>
+    <t>2025-11-15T17:14:08+01:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
Update to version 0.2.0
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-retina-conclusioncode-cs.xlsx
+++ b/docs/CodeSystem-retina-conclusioncode-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="59">
   <si>
     <t>Property</t>
   </si>
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.3</t>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>Grading Conclusion</t>
+    <t>Retina Conclusion</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-11-13T17:39:30+01:00</t>
+    <t>2025-11-30T22:57:21+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Codes describing where the external client has landed in its assessment of the examination. (1000-series)</t>
+    <t>Codes for the current or final conclusion of the grading process (1000-series).</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -120,7 +120,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>3</t>
+    <t>6</t>
   </si>
   <si>
     <t>Level</t>
@@ -141,19 +141,55 @@
     <t>1001</t>
   </si>
   <si>
-    <t>Grading completed</t>
+    <t>KI-gradering (basert på nåværende bilder)</t>
+  </si>
+  <si>
+    <t>This examination is waiting to be graded by the AI system.</t>
   </si>
   <si>
     <t>1002</t>
   </si>
   <si>
-    <t>To primary grading</t>
+    <t>Primærgradering (basert på nåværende bilder)</t>
+  </si>
+  <si>
+    <t>This examintions is waiting to be graded by a primary grader.</t>
   </si>
   <si>
     <t>1003</t>
   </si>
   <si>
-    <t>To secondary grading</t>
+    <t>Sekundærgradering (basert på nåværende bilder)</t>
+  </si>
+  <si>
+    <t>This examination is waiting to be graded by a secondary grader.</t>
+  </si>
+  <si>
+    <t>1004</t>
+  </si>
+  <si>
+    <t>Ny fotokontroll (primærgradering)</t>
+  </si>
+  <si>
+    <t>Patient should be scheduled for a new routine eye examination graded by primary grader or AI.</t>
+  </si>
+  <si>
+    <t>1005</t>
+  </si>
+  <si>
+    <t>Ny fotokontroll (sekundærgradering)</t>
+  </si>
+  <si>
+    <t>Patient should be scheduled for a new routine eye examination buty graded by secondary grader.</t>
+  </si>
+  <si>
+    <t>1006</t>
+  </si>
+  <si>
+    <t>Øyelegeundersøkelse (grunnet diabetisk retinopati)</t>
+  </si>
+  <si>
+    <t>Patient is leaving the screening program and should be referred to an ophthalmologist for further examination due to findings of diabetic retinopathy.</t>
   </si>
 </sst>
 </file>
@@ -463,7 +499,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -490,31 +526,79 @@
       <c r="C2" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" t="s" s="2">
+        <v>43</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="2">
         <v>40</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>44</v>
-      </c>
-      <c r="D3" s="2"/>
+        <v>45</v>
+      </c>
+      <c r="D3" t="s" s="2">
+        <v>46</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
         <v>40</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>46</v>
-      </c>
-      <c r="D4" s="2"/>
+        <v>48</v>
+      </c>
+      <c r="D4" t="s" s="2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>50</v>
+      </c>
+      <c r="C5" t="s" s="2">
+        <v>51</v>
+      </c>
+      <c r="D5" t="s" s="2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s" s="2">
+        <v>53</v>
+      </c>
+      <c r="C6" t="s" s="2">
+        <v>54</v>
+      </c>
+      <c r="D6" t="s" s="2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>56</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>57</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>58</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>